<commit_message>
Update Dominion Excel model without preferred stock table
</commit_message>
<xml_diff>
--- a/pitches/Dominion_Comparable_Company_Valuation.xlsx
+++ b/pitches/Dominion_Comparable_Company_Valuation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emory-my.sharepoint.com/personal/otstone_emory_edu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="211" documentId="8_{52DE5255-D58A-5A48-8D7E-98F4B21E82CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B553A14D-03BF-0548-813C-8CB7FAA5A9C0}"/>
+  <xr:revisionPtr revIDLastSave="212" documentId="8_{52DE5255-D58A-5A48-8D7E-98F4B21E82CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53EAA579-F1F0-A645-BB24-D096056332AB}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dominion Valuation" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="50">
   <si>
     <t>Comparable Companies Analysis</t>
   </si>
@@ -182,9 +182,6 @@
   </si>
   <si>
     <t>Market Data (as of September 18, 2026)</t>
-  </si>
-  <si>
-    <t>Preferred</t>
   </si>
   <si>
     <t>($ in millions, except per-share data)</t>
@@ -203,8 +200,8 @@
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@"/>
     <numFmt numFmtId="166" formatCode="#,##0.0\x"/>
     <numFmt numFmtId="167" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@"/>
-    <numFmt numFmtId="170" formatCode="_(\ #,##0.0_);_(\ \(#,##0.0\)_);_(\ &quot; - &quot;_)"/>
-    <numFmt numFmtId="178" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="_(\ #,##0.0_);_(\ \(#,##0.0\)_);_(\ &quot; - &quot;_)"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -489,11 +486,6 @@
     <xf numFmtId="166" fontId="3" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -507,22 +499,27 @@
     <xf numFmtId="165" fontId="3" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="3" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="3" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="39" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="39" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -762,7 +759,7 @@
   <sheetData>
     <row r="1" spans="2:16" ht="16" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:16" ht="24" x14ac:dyDescent="0.3">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="43" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="3"/>
@@ -781,8 +778,8 @@
       <c r="P2" s="3"/>
     </row>
     <row r="3" spans="2:16" ht="16" x14ac:dyDescent="0.2">
-      <c r="B3" s="53" t="s">
-        <v>49</v>
+      <c r="B3" s="50" t="s">
+        <v>48</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -802,25 +799,25 @@
     <row r="4" spans="2:16" ht="16" x14ac:dyDescent="0.2">
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="34"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="52"/>
+      <c r="H4" s="53"/>
       <c r="I4" s="4"/>
-      <c r="J4" s="32" t="s">
+      <c r="J4" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="K4" s="33"/>
-      <c r="L4" s="34"/>
+      <c r="K4" s="52"/>
+      <c r="L4" s="53"/>
       <c r="M4" s="4"/>
-      <c r="N4" s="32" t="s">
+      <c r="N4" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="O4" s="33"/>
-      <c r="P4" s="34"/>
+      <c r="O4" s="52"/>
+      <c r="P4" s="53"/>
     </row>
     <row r="5" spans="2:16" ht="34" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
@@ -883,50 +880,50 @@
       <c r="P6" s="10"/>
     </row>
     <row r="7" spans="2:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="39" t="s">
-        <v>50</v>
-      </c>
-      <c r="C7" s="40" t="s">
+      <c r="B7" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="47">
+      <c r="D7" s="44">
         <v>63.58</v>
       </c>
-      <c r="E7" s="48">
+      <c r="E7" s="45">
         <v>879.5</v>
       </c>
-      <c r="F7" s="41">
+      <c r="F7" s="38">
         <f>D7*E7</f>
         <v>55918.61</v>
       </c>
-      <c r="G7" s="48">
+      <c r="G7" s="45">
         <v>53634</v>
       </c>
-      <c r="H7" s="41">
+      <c r="H7" s="38">
         <f>F7+G7</f>
         <v>109552.61</v>
       </c>
-      <c r="I7" s="42"/>
-      <c r="J7" s="48">
+      <c r="I7" s="39"/>
+      <c r="J7" s="45">
         <v>18119</v>
       </c>
-      <c r="K7" s="48">
+      <c r="K7" s="45">
         <v>8341</v>
       </c>
-      <c r="L7" s="49">
+      <c r="L7" s="46">
         <v>2534</v>
       </c>
-      <c r="M7" s="43"/>
-      <c r="N7" s="44">
+      <c r="M7" s="40"/>
+      <c r="N7" s="41">
         <f>H7/J7</f>
         <v>6.0462834593520611</v>
       </c>
-      <c r="O7" s="44">
+      <c r="O7" s="41">
         <f>H7/K7</f>
         <v>13.134229708668025</v>
       </c>
-      <c r="P7" s="45">
-        <f>F7/L7</f>
+      <c r="P7" s="42">
+        <f t="shared" ref="P7:P17" si="0">F7/L7</f>
         <v>22.067328334648778</v>
       </c>
     </row>
@@ -937,44 +934,44 @@
       <c r="C8" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="50">
+      <c r="D8" s="47">
         <v>128.52000000000001</v>
       </c>
-      <c r="E8" s="51">
+      <c r="E8" s="48">
         <v>208.1</v>
       </c>
       <c r="F8" s="23">
         <f>D8*E8</f>
         <v>26745.012000000002</v>
       </c>
-      <c r="G8" s="51">
+      <c r="G8" s="48">
         <v>27798</v>
       </c>
-      <c r="H8" s="41">
-        <f t="shared" ref="H8:H17" si="0">F8+G8</f>
+      <c r="H8" s="38">
+        <f t="shared" ref="H8:H17" si="1">F8+G8</f>
         <v>54543.012000000002</v>
       </c>
       <c r="I8" s="28"/>
-      <c r="J8" s="51">
+      <c r="J8" s="48">
         <v>16465</v>
       </c>
-      <c r="K8" s="51">
+      <c r="K8" s="48">
         <v>3617</v>
       </c>
-      <c r="L8" s="52">
+      <c r="L8" s="49">
         <v>1317</v>
       </c>
       <c r="M8" s="31"/>
       <c r="N8" s="29">
-        <f t="shared" ref="N8:N17" si="1">H8/J8</f>
+        <f t="shared" ref="N8:N17" si="2">H8/J8</f>
         <v>3.3126639538414819</v>
       </c>
       <c r="O8" s="29">
-        <f t="shared" ref="O8:O17" si="2">H8/K8</f>
+        <f t="shared" ref="O8:O17" si="3">H8/K8</f>
         <v>15.079627315454797</v>
       </c>
       <c r="P8" s="30">
-        <f>F8/L8</f>
+        <f t="shared" si="0"/>
         <v>20.307526195899776</v>
       </c>
     </row>
@@ -985,44 +982,44 @@
       <c r="C9" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="50">
+      <c r="D9" s="47">
         <v>42.07</v>
       </c>
-      <c r="E9" s="51">
+      <c r="E9" s="48">
         <v>1032.3</v>
       </c>
       <c r="F9" s="23">
-        <f t="shared" ref="F9:F17" si="3">D9*E9</f>
+        <f t="shared" ref="F9:F17" si="4">D9*E9</f>
         <v>43428.860999999997</v>
       </c>
-      <c r="G9" s="51">
+      <c r="G9" s="48">
         <v>50860</v>
       </c>
-      <c r="H9" s="41">
-        <f t="shared" si="0"/>
+      <c r="H9" s="38">
+        <f t="shared" si="1"/>
         <v>94288.861000000004</v>
       </c>
       <c r="I9" s="12"/>
-      <c r="J9" s="51">
+      <c r="J9" s="48">
         <v>25326</v>
       </c>
-      <c r="K9" s="51">
+      <c r="K9" s="48">
         <v>8355</v>
       </c>
-      <c r="L9" s="52">
+      <c r="L9" s="49">
         <v>2783</v>
       </c>
       <c r="M9" s="13"/>
       <c r="N9" s="29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.7230064360736006</v>
       </c>
       <c r="O9" s="29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>11.285321484141233</v>
       </c>
       <c r="P9" s="30">
-        <f>F9/L9</f>
+        <f t="shared" si="0"/>
         <v>15.605052461372619</v>
       </c>
     </row>
@@ -1033,44 +1030,44 @@
       <c r="C10" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="50">
+      <c r="D10" s="47">
         <v>105.43</v>
       </c>
-      <c r="E10" s="51">
+      <c r="E10" s="48">
         <v>369.8</v>
       </c>
       <c r="F10" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>38988.014000000003</v>
       </c>
-      <c r="G10" s="51">
+      <c r="G10" s="48">
         <v>26850</v>
       </c>
-      <c r="H10" s="41">
-        <f t="shared" si="0"/>
+      <c r="H10" s="38">
+        <f t="shared" si="1"/>
         <v>65838.013999999996</v>
       </c>
       <c r="I10" s="12"/>
-      <c r="J10" s="51">
+      <c r="J10" s="48">
         <v>17689</v>
       </c>
-      <c r="K10" s="51">
+      <c r="K10" s="48">
         <v>6162</v>
       </c>
-      <c r="L10" s="52">
+      <c r="L10" s="49">
         <v>2217</v>
       </c>
       <c r="M10" s="13"/>
       <c r="N10" s="29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.7219748996551525</v>
       </c>
       <c r="O10" s="29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10.68452028562155</v>
       </c>
       <c r="P10" s="30">
-        <f>F10/L10</f>
+        <f t="shared" si="0"/>
         <v>17.585933243121335</v>
       </c>
     </row>
@@ -1081,44 +1078,44 @@
       <c r="C11" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="50">
+      <c r="D11" s="47">
         <v>69.77</v>
       </c>
-      <c r="E11" s="51">
+      <c r="E11" s="48">
         <v>498.4</v>
       </c>
       <c r="F11" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>34773.367999999995</v>
       </c>
-      <c r="G11" s="51">
+      <c r="G11" s="48">
         <v>24486</v>
       </c>
-      <c r="H11" s="41">
-        <f t="shared" si="0"/>
+      <c r="H11" s="38">
+        <f t="shared" si="1"/>
         <v>59259.367999999995</v>
       </c>
       <c r="I11" s="12"/>
-      <c r="J11" s="51">
+      <c r="J11" s="48">
         <v>12543</v>
       </c>
-      <c r="K11" s="51">
+      <c r="K11" s="48">
         <v>4463</v>
       </c>
-      <c r="L11" s="52">
+      <c r="L11" s="49">
         <v>2012</v>
       </c>
       <c r="M11" s="13"/>
       <c r="N11" s="29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.7244971697361073</v>
       </c>
       <c r="O11" s="29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>13.277922473672417</v>
       </c>
       <c r="P11" s="30">
-        <f>F11/L11</f>
+        <f t="shared" si="0"/>
         <v>17.282986083499004</v>
       </c>
     </row>
@@ -1129,44 +1126,44 @@
       <c r="C12" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="50">
+      <c r="D12" s="47">
         <v>67.72</v>
       </c>
-      <c r="E12" s="51">
+      <c r="E12" s="48">
         <v>376.7</v>
       </c>
       <c r="F12" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>25510.124</v>
       </c>
-      <c r="G12" s="51">
+      <c r="G12" s="48">
         <v>27988.5</v>
       </c>
-      <c r="H12" s="41">
-        <f t="shared" si="0"/>
+      <c r="H12" s="38">
+        <f t="shared" si="1"/>
         <v>53498.623999999996</v>
       </c>
       <c r="I12" s="12"/>
-      <c r="J12" s="51">
+      <c r="J12" s="48">
         <v>13998.4</v>
       </c>
-      <c r="K12" s="51">
+      <c r="K12" s="48">
         <v>4933</v>
       </c>
-      <c r="L12" s="52">
+      <c r="L12" s="49">
         <v>1449.4</v>
       </c>
       <c r="M12" s="13"/>
       <c r="N12" s="29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.8217670590924677</v>
       </c>
       <c r="O12" s="29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10.845048449219542</v>
       </c>
       <c r="P12" s="30">
-        <f>F12/L12</f>
+        <f t="shared" si="0"/>
         <v>17.600471919414929</v>
       </c>
     </row>
@@ -1177,44 +1174,44 @@
       <c r="C13" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="50">
+      <c r="D13" s="47">
         <v>102.01</v>
       </c>
-      <c r="E13" s="51">
+      <c r="E13" s="48">
         <v>477.8</v>
       </c>
       <c r="F13" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>48740.378000000004</v>
       </c>
-      <c r="G13" s="51">
+      <c r="G13" s="48">
         <v>30772.3</v>
       </c>
-      <c r="H13" s="41">
-        <f t="shared" si="0"/>
+      <c r="H13" s="38">
+        <f t="shared" si="1"/>
         <v>79512.678</v>
       </c>
       <c r="I13" s="12"/>
-      <c r="J13" s="51">
+      <c r="J13" s="48">
         <v>13482.2</v>
       </c>
-      <c r="K13" s="51">
+      <c r="K13" s="48">
         <v>5538.1</v>
       </c>
-      <c r="L13" s="52">
+      <c r="L13" s="49">
         <v>1797.1</v>
       </c>
       <c r="M13" s="13"/>
       <c r="N13" s="29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>5.8976041002210318</v>
       </c>
       <c r="O13" s="29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>14.357392968707678</v>
       </c>
       <c r="P13" s="30">
-        <f>F13/L13</f>
+        <f t="shared" si="0"/>
         <v>27.121683823938572</v>
       </c>
     </row>
@@ -1225,44 +1222,44 @@
       <c r="C14" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="50">
+      <c r="D14" s="47">
         <v>81.31</v>
       </c>
-      <c r="E14" s="51">
+      <c r="E14" s="48">
         <v>653.9</v>
       </c>
       <c r="F14" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>53168.608999999997</v>
       </c>
-      <c r="G14" s="51">
+      <c r="G14" s="48">
         <v>36616</v>
       </c>
-      <c r="H14" s="41">
-        <f t="shared" si="0"/>
+      <c r="H14" s="38">
+        <f t="shared" si="1"/>
         <v>89784.608999999997</v>
       </c>
       <c r="I14" s="12"/>
-      <c r="J14" s="51">
+      <c r="J14" s="48">
         <v>13552</v>
       </c>
-      <c r="K14" s="51">
+      <c r="K14" s="48">
         <v>5874</v>
       </c>
-      <c r="L14" s="52">
+      <c r="L14" s="49">
         <v>2280</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6.6251925177095625</v>
       </c>
       <c r="O14" s="29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>15.28508835546476</v>
       </c>
       <c r="P14" s="30">
-        <f>F14/L14</f>
+        <f t="shared" si="0"/>
         <v>23.319565350877191</v>
       </c>
     </row>
@@ -1273,44 +1270,44 @@
       <c r="C15" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="50">
+      <c r="D15" s="47">
         <v>120</v>
       </c>
-      <c r="E15" s="51">
+      <c r="E15" s="48">
         <v>544.4</v>
       </c>
       <c r="F15" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>65328</v>
       </c>
-      <c r="G15" s="51">
+      <c r="G15" s="48">
         <v>52922</v>
       </c>
-      <c r="H15" s="41">
-        <f t="shared" si="0"/>
+      <c r="H15" s="38">
+        <f t="shared" si="1"/>
         <v>118250</v>
       </c>
       <c r="I15" s="12"/>
-      <c r="J15" s="51">
+      <c r="J15" s="48">
         <v>22791</v>
       </c>
-      <c r="K15" s="51">
+      <c r="K15" s="48">
         <v>9029</v>
       </c>
-      <c r="L15" s="52">
+      <c r="L15" s="49">
         <v>3141</v>
       </c>
       <c r="M15" s="13"/>
       <c r="N15" s="29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>5.1884515817647321</v>
       </c>
       <c r="O15" s="29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>13.096688448333149</v>
       </c>
       <c r="P15" s="30">
-        <f>F15/L15</f>
+        <f t="shared" si="0"/>
         <v>20.798471824259789</v>
       </c>
     </row>
@@ -1321,44 +1318,44 @@
       <c r="C16" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="50">
+      <c r="D16" s="47">
         <v>85.52</v>
       </c>
-      <c r="E16" s="51">
+      <c r="E16" s="48">
         <v>1150.4000000000001</v>
       </c>
       <c r="F16" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>98382.207999999999</v>
       </c>
-      <c r="G16" s="51">
+      <c r="G16" s="48">
         <v>74103</v>
       </c>
-      <c r="H16" s="41">
-        <f t="shared" si="0"/>
+      <c r="H16" s="38">
+        <f t="shared" si="1"/>
         <v>172485.20799999998</v>
       </c>
       <c r="I16" s="12"/>
-      <c r="J16" s="51">
+      <c r="J16" s="48">
         <v>30179</v>
       </c>
-      <c r="K16" s="51">
+      <c r="K16" s="48">
         <v>14258</v>
       </c>
-      <c r="L16" s="52">
+      <c r="L16" s="49">
         <v>4658</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>5.7154050167334898</v>
       </c>
       <c r="O16" s="29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>12.097433581147424</v>
       </c>
       <c r="P16" s="30">
-        <f>F16/L16</f>
+        <f t="shared" si="0"/>
         <v>21.121126663804208</v>
       </c>
     </row>
@@ -1369,44 +1366,44 @@
       <c r="C17" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="50">
+      <c r="D17" s="47">
         <v>103.17</v>
       </c>
-      <c r="E17" s="51">
+      <c r="E17" s="48">
         <v>325.8</v>
       </c>
       <c r="F17" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>33612.786</v>
       </c>
-      <c r="G17" s="51">
+      <c r="G17" s="48">
         <v>22973.200000000001</v>
       </c>
-      <c r="H17" s="41">
-        <f t="shared" si="0"/>
+      <c r="H17" s="38">
+        <f t="shared" si="1"/>
         <v>56585.986000000004</v>
       </c>
       <c r="I17" s="12"/>
-      <c r="J17" s="51">
+      <c r="J17" s="48">
         <v>10137.4</v>
       </c>
-      <c r="K17" s="51">
+      <c r="K17" s="48">
         <v>3965.2</v>
       </c>
-      <c r="L17" s="52">
+      <c r="L17" s="49">
         <v>1691.5</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>5.5819032493538785</v>
       </c>
       <c r="O17" s="29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>14.270651165136691</v>
       </c>
       <c r="P17" s="30">
-        <f>F17/L17</f>
+        <f t="shared" si="0"/>
         <v>19.871584983742242</v>
       </c>
     </row>
@@ -1447,11 +1444,11 @@
         <v>6.6251925177095625</v>
       </c>
       <c r="O19" s="14">
-        <f t="shared" ref="O19:P19" si="4">MAX(O8:O17)</f>
+        <f t="shared" ref="O19:P19" si="5">MAX(O8:O17)</f>
         <v>15.28508835546476</v>
       </c>
       <c r="P19" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>27.121683823938572</v>
       </c>
     </row>
@@ -1475,11 +1472,11 @@
         <v>5.6820295748885865</v>
       </c>
       <c r="O20" s="14">
-        <f t="shared" ref="O20:P20" si="5">QUARTILE(O8:O17,3)</f>
+        <f t="shared" ref="O20:P20" si="6">QUARTILE(O8:O17,3)</f>
         <v>14.335707517814932</v>
       </c>
       <c r="P20" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>21.040462953918102</v>
       </c>
     </row>
@@ -1503,11 +1500,11 @@
         <v>4.8312465984181507</v>
       </c>
       <c r="O21" s="16">
-        <f t="shared" ref="O21:P21" si="6">AVERAGE(O8:O17)</f>
+        <f t="shared" ref="O21:P21" si="7">AVERAGE(O8:O17)</f>
         <v>13.027969452689925</v>
       </c>
       <c r="P21" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>20.061440254992966</v>
       </c>
     </row>
@@ -1531,11 +1528,11 @@
         <v>4.9564743757504193</v>
       </c>
       <c r="O22" s="16">
-        <f t="shared" ref="O22:P22" si="7">MEDIAN(O8:O17)</f>
+        <f t="shared" ref="O22:P22" si="8">MEDIAN(O8:O17)</f>
         <v>13.187305461002783</v>
       </c>
       <c r="P22" s="16">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>20.089555589821011</v>
       </c>
     </row>
@@ -1559,11 +1556,11 @@
         <v>3.7476965918283174</v>
       </c>
       <c r="O23" s="14">
-        <f t="shared" ref="O23:P23" si="8">QUARTILE(O8:O17,1)</f>
+        <f t="shared" ref="O23:P23" si="9">QUARTILE(O8:O17,1)</f>
         <v>11.488349508392782</v>
       </c>
       <c r="P23" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>17.589567912194735</v>
       </c>
     </row>
@@ -1587,11 +1584,11 @@
         <v>3.3126639538414819</v>
       </c>
       <c r="O24" s="14">
-        <f t="shared" ref="O24:P24" si="9">MIN(O8:O17)</f>
+        <f t="shared" ref="O24:P24" si="10">MIN(O8:O17)</f>
         <v>10.68452028562155</v>
       </c>
       <c r="P24" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>15.605052461372619</v>
       </c>
     </row>
@@ -1794,175 +1791,127 @@
     <row r="35" spans="2:9" ht="16" x14ac:dyDescent="0.2">
       <c r="D35" s="18"/>
       <c r="E35" s="18"/>
-      <c r="F35" s="35"/>
+      <c r="F35" s="32"/>
     </row>
     <row r="40" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="36"/>
-      <c r="C40" s="36"/>
-      <c r="D40" s="36"/>
-      <c r="F40" s="36" t="s">
-        <v>3</v>
-      </c>
-      <c r="G40" s="36" t="s">
-        <v>48</v>
-      </c>
+      <c r="B40" s="33"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="33"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="33"/>
     </row>
     <row r="41" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="37"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="38"/>
-      <c r="F41" s="37" t="s">
-        <v>42</v>
-      </c>
-      <c r="G41" s="37">
-        <v>991</v>
-      </c>
+      <c r="B41" s="34"/>
+      <c r="C41" s="34"/>
+      <c r="D41" s="35"/>
+      <c r="F41" s="34"/>
+      <c r="G41" s="34"/>
     </row>
     <row r="42" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="37"/>
-      <c r="C42" s="37"/>
-      <c r="D42" s="37"/>
-      <c r="F42" s="37" t="s">
-        <v>25</v>
-      </c>
-      <c r="G42" s="37">
-        <v>0</v>
-      </c>
-      <c r="H42" s="36"/>
-      <c r="I42" s="36"/>
+      <c r="B42" s="34"/>
+      <c r="C42" s="34"/>
+      <c r="D42" s="34"/>
+      <c r="F42" s="34"/>
+      <c r="G42" s="34"/>
+      <c r="H42" s="33"/>
+      <c r="I42" s="33"/>
     </row>
     <row r="43" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="37"/>
-      <c r="C43" s="37"/>
-      <c r="D43" s="37"/>
-      <c r="F43" s="37" t="s">
-        <v>26</v>
-      </c>
-      <c r="G43" s="37">
-        <v>0</v>
-      </c>
-      <c r="H43" s="37"/>
-      <c r="I43" s="38"/>
+      <c r="B43" s="34"/>
+      <c r="C43" s="34"/>
+      <c r="D43" s="34"/>
+      <c r="F43" s="34"/>
+      <c r="G43" s="34"/>
+      <c r="H43" s="34"/>
+      <c r="I43" s="35"/>
     </row>
     <row r="44" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="37"/>
-      <c r="C44" s="37"/>
-      <c r="D44" s="37"/>
-      <c r="F44" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="G44" s="37">
-        <v>0</v>
-      </c>
-      <c r="H44" s="37"/>
-      <c r="I44" s="38"/>
+      <c r="B44" s="34"/>
+      <c r="C44" s="34"/>
+      <c r="D44" s="34"/>
+      <c r="F44" s="34"/>
+      <c r="G44" s="34"/>
+      <c r="H44" s="34"/>
+      <c r="I44" s="35"/>
     </row>
     <row r="45" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="37"/>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-      <c r="F45" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="G45" s="37">
-        <v>0</v>
-      </c>
-      <c r="H45" s="37"/>
-      <c r="I45" s="38"/>
+      <c r="B45" s="34"/>
+      <c r="C45" s="34"/>
+      <c r="D45" s="34"/>
+      <c r="F45" s="34"/>
+      <c r="G45" s="34"/>
+      <c r="H45" s="34"/>
+      <c r="I45" s="35"/>
     </row>
     <row r="46" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="37"/>
-      <c r="C46" s="37"/>
-      <c r="D46" s="37"/>
-      <c r="F46" s="37" t="s">
-        <v>29</v>
-      </c>
-      <c r="G46" s="37">
-        <v>0</v>
-      </c>
-      <c r="H46" s="37"/>
-      <c r="I46" s="38"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="34"/>
+      <c r="D46" s="34"/>
+      <c r="F46" s="34"/>
+      <c r="G46" s="34"/>
+      <c r="H46" s="34"/>
+      <c r="I46" s="35"/>
     </row>
     <row r="47" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="37"/>
-      <c r="C47" s="37"/>
-      <c r="D47" s="37"/>
-      <c r="F47" s="37" t="s">
-        <v>30</v>
-      </c>
-      <c r="G47" s="37">
-        <v>0</v>
-      </c>
-      <c r="H47" s="37"/>
-      <c r="I47" s="38"/>
+      <c r="B47" s="34"/>
+      <c r="C47" s="34"/>
+      <c r="D47" s="34"/>
+      <c r="F47" s="34"/>
+      <c r="G47" s="34"/>
+      <c r="H47" s="34"/>
+      <c r="I47" s="35"/>
     </row>
     <row r="48" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="37"/>
-      <c r="C48" s="37"/>
-      <c r="D48" s="38"/>
-      <c r="F48" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="G48" s="37">
-        <v>0</v>
-      </c>
-      <c r="H48" s="37"/>
-      <c r="I48" s="38"/>
+      <c r="B48" s="34"/>
+      <c r="C48" s="34"/>
+      <c r="D48" s="35"/>
+      <c r="F48" s="34"/>
+      <c r="G48" s="34"/>
+      <c r="H48" s="34"/>
+      <c r="I48" s="35"/>
     </row>
     <row r="49" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="37"/>
-      <c r="C49" s="37"/>
-      <c r="D49" s="38"/>
-      <c r="F49" s="37" t="s">
-        <v>32</v>
-      </c>
-      <c r="G49" s="37">
-        <v>0</v>
-      </c>
-      <c r="H49" s="37"/>
-      <c r="I49" s="38"/>
+      <c r="B49" s="34"/>
+      <c r="C49" s="34"/>
+      <c r="D49" s="35"/>
+      <c r="F49" s="34"/>
+      <c r="G49" s="34"/>
+      <c r="H49" s="34"/>
+      <c r="I49" s="35"/>
     </row>
     <row r="50" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B50" s="37"/>
-      <c r="C50" s="37"/>
-      <c r="D50" s="38"/>
-      <c r="F50" s="37" t="s">
-        <v>33</v>
-      </c>
-      <c r="G50" s="37">
-        <v>0</v>
-      </c>
-      <c r="H50" s="37"/>
-      <c r="I50" s="38"/>
+      <c r="B50" s="34"/>
+      <c r="C50" s="34"/>
+      <c r="D50" s="35"/>
+      <c r="F50" s="34"/>
+      <c r="G50" s="34"/>
+      <c r="H50" s="34"/>
+      <c r="I50" s="35"/>
     </row>
     <row r="51" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="25"/>
       <c r="C51" s="25"/>
       <c r="D51" s="24"/>
-      <c r="F51" s="37" t="s">
-        <v>34</v>
-      </c>
-      <c r="G51" s="37">
-        <v>0</v>
-      </c>
-      <c r="H51" s="37"/>
-      <c r="I51" s="38"/>
+      <c r="F51" s="34"/>
+      <c r="G51" s="34"/>
+      <c r="H51" s="34"/>
+      <c r="I51" s="35"/>
     </row>
     <row r="52" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="25"/>
       <c r="C52" s="25"/>
       <c r="D52" s="24"/>
-      <c r="G52" s="37"/>
-      <c r="H52" s="37"/>
-      <c r="I52" s="38"/>
+      <c r="G52" s="34"/>
+      <c r="H52" s="34"/>
+      <c r="I52" s="35"/>
     </row>
     <row r="53" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B53" s="25"/>
       <c r="C53" s="25"/>
       <c r="D53" s="24"/>
-      <c r="G53" s="37"/>
-      <c r="H53" s="37"/>
-      <c r="I53" s="38"/>
+      <c r="G53" s="34"/>
+      <c r="H53" s="34"/>
+      <c r="I53" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>